<commit_message>
WIP checkpoint 2026-08-24: skill v2, portfolio architecture, eval cleanup, new research docs
</commit_message>
<xml_diff>
--- a/data/raw/etf-evaluation-framework.xlsx
+++ b/data/raw/etf-evaluation-framework.xlsx
@@ -1,26 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eduardofgiovannini/Documents/Interactive_Brokers/ETF’S main Metrics/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eduardofgiovannini/Documents/GitHub/Global_Retirement_ETF_Strategy/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36FFCE32-FC10-5F4C-A3E8-61E400A62D55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B099C83B-EB87-4243-8CF1-EB2636FB9B19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="3980" windowWidth="76800" windowHeight="20980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22420" yWindow="17520" windowWidth="25600" windowHeight="14800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="ETF Evaluation Framework" sheetId="1" r:id="rId1"/>
+    <sheet name="5-Minute Brief" sheetId="2" r:id="rId1"/>
+    <sheet name="ETF Evaluation Framework" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="168">
   <si>
     <t>Metric</t>
   </si>
@@ -218,13 +219,319 @@
   </si>
   <si>
     <t>Use to size risk across different asset classes (e.g., equities vs. bonds), not to differentiate similar index ETFs.</t>
+  </si>
+  <si>
+    <t>ETF Evaluation Framework — 5-Minute Brief</t>
+  </si>
+  <si>
+    <t>Decision-first guide to selecting broad-market ETFs, distilled from all 14 metrics in the framework.</t>
+  </si>
+  <si>
+    <t>BOTTOM LINE</t>
+  </si>
+  <si>
+    <t>Start with tax domicile and index scope; then compare realized costs and execution quality. Portfolio exposures come next, while yield, AUM, trailing returns, and volatility are supporting checks—not primary selection criteria. For non-U.S. investors, domicile can outweigh small fee differences because it affects estate-tax exposure and dividend withholding.</t>
+  </si>
+  <si>
+    <t>DECISION ORDER — WHAT TO CHECK FIRST</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Topic</t>
+  </si>
+  <si>
+    <t>What to establish</t>
+  </si>
+  <si>
+    <t>Practical rule</t>
+  </si>
+  <si>
+    <t>Framework tier</t>
+  </si>
+  <si>
+    <t>Decision role</t>
+  </si>
+  <si>
+    <t>Eligibility &amp; structure</t>
+  </si>
+  <si>
+    <t>Domicile, exact benchmark/cap scope, issuer, inception</t>
+  </si>
+  <si>
+    <t>Resolve tax/legal fit and confirm exactly what the fund owns before comparing prices.</t>
+  </si>
+  <si>
+    <t>Tier 1</t>
+  </si>
+  <si>
+    <t>Dealbreaker</t>
+  </si>
+  <si>
+    <t>True ownership cost</t>
+  </si>
+  <si>
+    <t>Tracking difference, expense ratio, spread, NAV premium/discount, turnover</t>
+  </si>
+  <si>
+    <t>Prefer tracking difference near 0%; broad-market fee &lt;0.10%; turnover &lt;10%, typically &lt;5%.</t>
+  </si>
+  <si>
+    <t>Tier 2</t>
+  </si>
+  <si>
+    <t>Core comparison</t>
+  </si>
+  <si>
+    <t>Portfolio reality</t>
+  </si>
+  <si>
+    <t>Country/region weight, top-10 concentration, P/E and P/B</t>
+  </si>
+  <si>
+    <t>Check U.S. concentration, mega-cap overlap, and whether valuations fit your risk expectations.</t>
+  </si>
+  <si>
+    <t>Tier 3</t>
+  </si>
+  <si>
+    <t>Exposure check</t>
+  </si>
+  <si>
+    <t>Income &amp; viability</t>
+  </si>
+  <si>
+    <t>Yield/distribution schedule and AUM</t>
+  </si>
+  <si>
+    <t>Match cash-flow needs; prefer core funds with &gt;$500M–$1B+ AUM.</t>
+  </si>
+  <si>
+    <t>Tier 4</t>
+  </si>
+  <si>
+    <t>Supporting check</t>
+  </si>
+  <si>
+    <t>Historical sanity check</t>
+  </si>
+  <si>
+    <t>1Y/3Y/5Y returns, volatility, maximum drawdown</t>
+  </si>
+  <si>
+    <t>Use to confirm expected behavior—not to rank near-identical index ETFs.</t>
+  </si>
+  <si>
+    <t>Tier 5</t>
+  </si>
+  <si>
+    <t>Do not over-weight</t>
+  </si>
+  <si>
+    <t>TOP HIGHLIGHTS</t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t>Highlight</t>
+  </si>
+  <si>
+    <t>Why it matters</t>
+  </si>
+  <si>
+    <t>Implication</t>
+  </si>
+  <si>
+    <t>Metric(s)</t>
+  </si>
+  <si>
+    <t>Domicile is the highest-leverage field</t>
+  </si>
+  <si>
+    <t>For non-U.S. investors it can affect U.S. estate-tax exposure and dividend withholding leakage.</t>
+  </si>
+  <si>
+    <t>Compare U.S.-domiciled funds with Irish-domiciled UCITS alternatives before choosing.</t>
+  </si>
+  <si>
+    <t>Critical</t>
+  </si>
+  <si>
+    <t>Fund names can hide material scope differences</t>
+  </si>
+  <si>
+    <t>“Global” or “World” may cover large/mid caps only or include small caps and thousands more holdings.</t>
+  </si>
+  <si>
+    <t>Read the exact index methodology; do not use holdings count alone as a quality score.</t>
+  </si>
+  <si>
+    <t>Tracking difference is more complete than the stated fee</t>
+  </si>
+  <si>
+    <t>It captures fees net of lending revenue plus cash drag and other implementation effects.</t>
+  </si>
+  <si>
+    <t>Compare 3–5-year tracking difference, aiming near 0.00% or slightly positive.</t>
+  </si>
+  <si>
+    <t>4–5</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Execution costs stack</t>
+  </si>
+  <si>
+    <t>Bid-ask spread plus NAV premium/discount can create an immediate entry/exit surcharge.</t>
+  </si>
+  <si>
+    <t>Check live spreads and premiums during market hours, especially for smaller funds.</t>
+  </si>
+  <si>
+    <t>“Global” remains U.S.-heavy</t>
+  </si>
+  <si>
+    <t>Market-cap-weighted global ETFs may hold 60%+ in U.S. equities and concentrate in mega-cap technology.</t>
+  </si>
+  <si>
+    <t>Review regional weight and top-10 overlap with other holdings.</t>
+  </si>
+  <si>
+    <t>8–10</t>
+  </si>
+  <si>
+    <t>YOUR ACTION CHECKLIST</t>
+  </si>
+  <si>
+    <t>Step</t>
+  </si>
+  <si>
+    <t>Action</t>
+  </si>
+  <si>
+    <t>Question to answer</t>
+  </si>
+  <si>
+    <t>Target / evidence</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Define tax eligibility</t>
+  </si>
+  <si>
+    <t>Is a U.S.-domiciled ETF tax-advantaged in your jurisdiction?</t>
+  </si>
+  <si>
+    <t>If not, evaluate Irish-domiciled UCITS equivalents.</t>
+  </si>
+  <si>
+    <t>□</t>
+  </si>
+  <si>
+    <t>Choose desired market scope</t>
+  </si>
+  <si>
+    <t>Do you want large/mid cap or all-cap exposure including small caps?</t>
+  </si>
+  <si>
+    <t>Match the exact benchmark rules to the intended reach.</t>
+  </si>
+  <si>
+    <t>Confirm operational quality</t>
+  </si>
+  <si>
+    <t>Is the issuer established and the product likely to persist?</t>
+  </si>
+  <si>
+    <t>Favor top-tier issuers; scrutinize niche/new funds more strictly.</t>
+  </si>
+  <si>
+    <t>Compare realized cost</t>
+  </si>
+  <si>
+    <t>How closely has each fund tracked its benchmark over 3–5 years?</t>
+  </si>
+  <si>
+    <t>Tracking difference near 0.00% or slightly positive; fee &lt;0.10% for broad market.</t>
+  </si>
+  <si>
+    <t>Check trade execution</t>
+  </si>
+  <si>
+    <t>What are the live spread and NAV premium/discount?</t>
+  </si>
+  <si>
+    <t>Trade during market hours; avoid stacked execution costs.</t>
+  </si>
+  <si>
+    <t>Audit portfolio overlap</t>
+  </si>
+  <si>
+    <t>Are U.S., top-10, or mega-cap tech exposures excessive across your total portfolio?</t>
+  </si>
+  <si>
+    <t>Review regional weights and overlap with stocks or U.S. tech ETFs.</t>
+  </si>
+  <si>
+    <t>Run final supporting checks</t>
+  </si>
+  <si>
+    <t>Do distributions suit cash needs, is AUM adequate, and does risk behavior look normal?</t>
+  </si>
+  <si>
+    <t>Prefer &gt;$500M–$1B+ AUM; use returns/drawdown only as sanity checks.</t>
+  </si>
+  <si>
+    <t>11–14</t>
+  </si>
+  <si>
+    <t>METRIC MAP — ALL 14 ITEMS</t>
+  </si>
+  <si>
+    <t>Main question</t>
+  </si>
+  <si>
+    <t>Default interpretation</t>
+  </si>
+  <si>
+    <t>Target / guidance</t>
+  </si>
+  <si>
+    <t>Weight</t>
+  </si>
+  <si>
+    <t>Dealbreakers</t>
+  </si>
+  <si>
+    <t>Real Costs</t>
+  </si>
+  <si>
+    <t>Portfolio Reality</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Income Mechanics</t>
+  </si>
+  <si>
+    <t>Supporting</t>
+  </si>
+  <si>
+    <t>Sanity Checks</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -249,16 +556,105 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FF666666"/>
+      <name val="Aptos"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF17365D"/>
+      <name val="Aptos"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF17365D"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2F75B5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9EAF7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF5B9BD5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2F0D9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF7F9FC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -281,11 +677,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -295,6 +700,93 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -310,6 +802,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -650,6 +1146,852 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1E637C0-420D-EF48-AD12-DBA6553085ED}">
+  <dimension ref="A1:F48"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="7" customWidth="1"/>
+    <col min="2" max="2" width="25.83203125" customWidth="1"/>
+    <col min="3" max="4" width="33.33203125" customWidth="1"/>
+    <col min="5" max="6" width="20.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+    </row>
+    <row r="2" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+    </row>
+    <row r="4" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+    </row>
+    <row r="5" spans="1:6" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" s="5"/>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+    </row>
+    <row r="7" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="45" x14ac:dyDescent="0.2">
+      <c r="A9" s="15">
+        <v>1</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="F9" s="19" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="45" x14ac:dyDescent="0.2">
+      <c r="A10" s="24">
+        <v>2</v>
+      </c>
+      <c r="B10" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="C10" s="25" t="s">
+        <v>83</v>
+      </c>
+      <c r="D10" s="25" t="s">
+        <v>84</v>
+      </c>
+      <c r="E10" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="F10" s="26" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="45" x14ac:dyDescent="0.2">
+      <c r="A11" s="15">
+        <v>3</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="F11" s="19" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="30" x14ac:dyDescent="0.2">
+      <c r="A12" s="24">
+        <v>4</v>
+      </c>
+      <c r="B12" s="25" t="s">
+        <v>92</v>
+      </c>
+      <c r="C12" s="25" t="s">
+        <v>93</v>
+      </c>
+      <c r="D12" s="25" t="s">
+        <v>94</v>
+      </c>
+      <c r="E12" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="F12" s="26" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="30" x14ac:dyDescent="0.2">
+      <c r="A13" s="16">
+        <v>5</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="E13" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="F13" s="20" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" s="17"/>
+      <c r="B14" s="12"/>
+      <c r="C14" s="12"/>
+      <c r="D14" s="12"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="31"/>
+    </row>
+    <row r="15" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A15" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="B15" s="32"/>
+      <c r="C15" s="32"/>
+      <c r="D15" s="32"/>
+      <c r="E15" s="33"/>
+      <c r="F15" s="33"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="D16" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="45" x14ac:dyDescent="0.2">
+      <c r="A17" s="15">
+        <v>1</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="E17" s="15">
+        <v>1</v>
+      </c>
+      <c r="F17" s="21" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="45" x14ac:dyDescent="0.2">
+      <c r="A18" s="24">
+        <v>2</v>
+      </c>
+      <c r="B18" s="25" t="s">
+        <v>112</v>
+      </c>
+      <c r="C18" s="25" t="s">
+        <v>113</v>
+      </c>
+      <c r="D18" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="E18" s="24">
+        <v>2</v>
+      </c>
+      <c r="F18" s="26" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="45" x14ac:dyDescent="0.2">
+      <c r="A19" s="15">
+        <v>3</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="E19" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="F19" s="21" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="45" x14ac:dyDescent="0.2">
+      <c r="A20" s="24">
+        <v>4</v>
+      </c>
+      <c r="B20" s="25" t="s">
+        <v>120</v>
+      </c>
+      <c r="C20" s="25" t="s">
+        <v>121</v>
+      </c>
+      <c r="D20" s="25" t="s">
+        <v>122</v>
+      </c>
+      <c r="E20" s="24">
+        <v>6</v>
+      </c>
+      <c r="F20" s="26" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="45" x14ac:dyDescent="0.2">
+      <c r="A21" s="16">
+        <v>5</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="E21" s="16" t="s">
+        <v>126</v>
+      </c>
+      <c r="F21" s="22" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A22" s="17"/>
+      <c r="B22" s="12"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="30"/>
+      <c r="F22" s="31"/>
+    </row>
+    <row r="23" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A23" s="18" t="s">
+        <v>127</v>
+      </c>
+      <c r="B23" s="32"/>
+      <c r="C23" s="32"/>
+      <c r="D23" s="32"/>
+      <c r="E23" s="33"/>
+      <c r="F23" s="33"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A24" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="B24" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="D24" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="E24" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="F24" s="11" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="30" x14ac:dyDescent="0.2">
+      <c r="A25" s="15">
+        <v>1</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="E25" s="15">
+        <v>1</v>
+      </c>
+      <c r="F25" s="19" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="30" x14ac:dyDescent="0.2">
+      <c r="A26" s="24">
+        <v>2</v>
+      </c>
+      <c r="B26" s="25" t="s">
+        <v>137</v>
+      </c>
+      <c r="C26" s="25" t="s">
+        <v>138</v>
+      </c>
+      <c r="D26" s="25" t="s">
+        <v>139</v>
+      </c>
+      <c r="E26" s="24">
+        <v>2</v>
+      </c>
+      <c r="F26" s="26" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="30" x14ac:dyDescent="0.2">
+      <c r="A27" s="15">
+        <v>3</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>140</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="D27" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="E27" s="15">
+        <v>3</v>
+      </c>
+      <c r="F27" s="19" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="30" x14ac:dyDescent="0.2">
+      <c r="A28" s="24">
+        <v>4</v>
+      </c>
+      <c r="B28" s="25" t="s">
+        <v>143</v>
+      </c>
+      <c r="C28" s="25" t="s">
+        <v>144</v>
+      </c>
+      <c r="D28" s="25" t="s">
+        <v>145</v>
+      </c>
+      <c r="E28" s="24" t="s">
+        <v>118</v>
+      </c>
+      <c r="F28" s="26" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="30" x14ac:dyDescent="0.2">
+      <c r="A29" s="15">
+        <v>5</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>146</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="D29" s="13" t="s">
+        <v>148</v>
+      </c>
+      <c r="E29" s="15">
+        <v>6</v>
+      </c>
+      <c r="F29" s="19" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="45" x14ac:dyDescent="0.2">
+      <c r="A30" s="24">
+        <v>6</v>
+      </c>
+      <c r="B30" s="25" t="s">
+        <v>149</v>
+      </c>
+      <c r="C30" s="25" t="s">
+        <v>150</v>
+      </c>
+      <c r="D30" s="25" t="s">
+        <v>151</v>
+      </c>
+      <c r="E30" s="24" t="s">
+        <v>126</v>
+      </c>
+      <c r="F30" s="26" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="45" x14ac:dyDescent="0.2">
+      <c r="A31" s="16">
+        <v>7</v>
+      </c>
+      <c r="B31" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="C31" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="D31" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="E31" s="16" t="s">
+        <v>155</v>
+      </c>
+      <c r="F31" s="20" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A32" s="17"/>
+      <c r="B32" s="12"/>
+      <c r="C32" s="12"/>
+      <c r="D32" s="12"/>
+      <c r="E32" s="30"/>
+      <c r="F32" s="31"/>
+    </row>
+    <row r="33" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A33" s="18" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33" s="32"/>
+      <c r="C33" s="32"/>
+      <c r="D33" s="32"/>
+      <c r="E33" s="33"/>
+      <c r="F33" s="33"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A34" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B34" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C34" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="D34" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="E34" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="F34" s="11" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="90" x14ac:dyDescent="0.2">
+      <c r="A35" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B35" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="C35" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="D35" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E35" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="F35" s="23" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="75" x14ac:dyDescent="0.2">
+      <c r="A36" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="B36" s="25" t="s">
+        <v>161</v>
+      </c>
+      <c r="C36" s="25" t="s">
+        <v>11</v>
+      </c>
+      <c r="D36" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="E36" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="F36" s="26" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="60" x14ac:dyDescent="0.2">
+      <c r="A37" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B37" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="C37" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D37" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="E37" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="F37" s="23" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="75" x14ac:dyDescent="0.2">
+      <c r="A38" s="24" t="s">
+        <v>18</v>
+      </c>
+      <c r="B38" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="C38" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="D38" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="E38" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="F38" s="26" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="60" x14ac:dyDescent="0.2">
+      <c r="A39" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="B39" s="13" t="s">
+        <v>162</v>
+      </c>
+      <c r="C39" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="D39" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="E39" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="F39" s="23" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="135" x14ac:dyDescent="0.2">
+      <c r="A40" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="B40" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="C40" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="D40" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="E40" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="F40" s="26" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="75" x14ac:dyDescent="0.2">
+      <c r="A41" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="B41" s="13" t="s">
+        <v>162</v>
+      </c>
+      <c r="C41" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="D41" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="E41" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="F41" s="23" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="90" x14ac:dyDescent="0.2">
+      <c r="A42" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="B42" s="25" t="s">
+        <v>163</v>
+      </c>
+      <c r="C42" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="D42" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="E42" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="F42" s="26" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="60" x14ac:dyDescent="0.2">
+      <c r="A43" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B43" s="13" t="s">
+        <v>163</v>
+      </c>
+      <c r="C43" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="D43" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="E43" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="F43" s="23" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="120" x14ac:dyDescent="0.2">
+      <c r="A44" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B44" s="25" t="s">
+        <v>163</v>
+      </c>
+      <c r="C44" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="D44" s="25" t="s">
+        <v>46</v>
+      </c>
+      <c r="E44" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="F44" s="26" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="90" x14ac:dyDescent="0.2">
+      <c r="A45" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="B45" s="13" t="s">
+        <v>165</v>
+      </c>
+      <c r="C45" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D45" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="E45" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="F45" s="23" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="90" x14ac:dyDescent="0.2">
+      <c r="A46" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="B46" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="C46" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="D46" s="25" t="s">
+        <v>55</v>
+      </c>
+      <c r="E46" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="F46" s="26" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="75" x14ac:dyDescent="0.2">
+      <c r="A47" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="B47" s="13" t="s">
+        <v>167</v>
+      </c>
+      <c r="C47" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="D47" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="E47" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="F47" s="23" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="165" x14ac:dyDescent="0.2">
+      <c r="A48" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="B48" s="28" t="s">
+        <v>167</v>
+      </c>
+      <c r="C48" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="D48" s="28" t="s">
+        <v>64</v>
+      </c>
+      <c r="E48" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="F48" s="29" t="s">
+        <v>166</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="A15:F15"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>

</xml_diff>